<commit_message>
draft-icl v1.2; add draft-pfc v1.0
- draft-icl: reference-sample row, annotation clearance, compact review card, print verification
- draft-pfc: BOM-to-PFC with HTML review and stdlib Excel export on a masked form
- Templates: strip author paths and printer settings (embedded user name)
- README: draft-pfc section and workflow diagram

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/draft-icl/processes/bending/template.xlsx
+++ b/draft-icl/processes/bending/template.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\users\greg.steenvoorden\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{1B7E24A2-4339-4EEE-968A-9D689B193CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="292" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -2312,7 +2307,7 @@
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.19685039370078741" footer="0.19685039370078741"/>
-  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;L&amp;9IXL Management System</oddFooter>
   </headerFooter>

</xml_diff>